<commit_message>
Add strategy evaluation dashboard updates'
</commit_message>
<xml_diff>
--- a/data/JFMP_RR.xlsx
+++ b/data/JFMP_RR.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pb0e\Downloads\git_dashboard\streamlit-test\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pb0e\Downloads\Phils Scripts\jfmp_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D17A3FB-F61D-4E86-A2D0-3AEA72C1E94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0D6C41-934C-4995-84B4-8BC70D121847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3216" yWindow="2556" windowWidth="17280" windowHeight="8976" activeTab="1" xr2:uid="{67390A52-5801-4610-A7E5-7A5F58273BD5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{67390A52-5801-4610-A7E5-7A5F58273BD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Murray Goldfields" sheetId="1" r:id="rId1"/>

</xml_diff>